<commit_message>
Preserve every policy row when expanding the Excel template
</commit_message>
<xml_diff>
--- a/docs/downloads/meta_india_reports_latest.xlsx
+++ b/docs/downloads/meta_india_reports_latest.xlsx
@@ -1069,7 +1069,7 @@
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Generated by Meta India low-request pipeline on 2026-10-08 17:06 UTC.</t>
+          <t>Generated by Meta India low-request pipeline on 2026-10-08 17:08 UTC.</t>
         </is>
       </c>
     </row>
@@ -77378,9 +77378,8 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K1656"/>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1658:K1658"/>
-    <mergeCell ref="A43:K43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add date-range spreadsheet explorer and automatic Pages deployment
</commit_message>
<xml_diff>
--- a/docs/downloads/meta_india_reports_latest.xlsx
+++ b/docs/downloads/meta_india_reports_latest.xlsx
@@ -201,7 +201,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Facebook: Content Actioned (AI) vs Grievances Received</a:t>
+              <a:t>Facebook: Content Actioned vs Grievances Received</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -347,7 +347,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Instagram: Content Actioned (AI) vs Grievances Received</a:t>
+              <a:t>Instagram: Content Actioned vs Grievances Received</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -481,11 +481,157 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Threads: Content Actioned vs Grievances Received</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Threads: Content Actioned</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Trend Charts'!$A$2:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trend Charts'!$G$2:$G$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Threads: Grievances Received</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Trend Charts'!$A$2:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trend Charts'!$H$2:$H$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Month</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Count</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
@@ -507,7 +653,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>25</row>
       <rowOff>0</rowOff>
@@ -522,6 +668,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1069,7 +1237,7 @@
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Generated by Meta India low-request pipeline on 2026-10-08 17:12 UTC.</t>
+          <t>Generated by Meta India low-request pipeline on 2026-10-08 17:29 UTC.</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4785,6 +4953,8 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="23.85" customHeight="1">
@@ -4818,6 +4988,16 @@
           <t>IG: Grievances Received</t>
         </is>
       </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Threads: Content Actioned</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Threads: Grievances Received</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -4836,6 +5016,8 @@
         <v>2031300</v>
       </c>
       <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -4858,6 +5040,8 @@
       <c r="F3" s="7" t="n">
         <v>265</v>
       </c>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -4880,6 +5064,8 @@
       <c r="F4" s="7" t="n">
         <v>106</v>
       </c>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -4902,6 +5088,8 @@
       <c r="F5" s="7" t="n">
         <v>418</v>
       </c>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -4924,6 +5112,8 @@
       <c r="F6" s="7" t="n">
         <v>414</v>
       </c>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -4946,6 +5136,8 @@
       <c r="F7" s="7" t="n">
         <v>1037</v>
       </c>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -4968,6 +5160,8 @@
       <c r="F8" s="7" t="n">
         <v>1050</v>
       </c>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -4990,6 +5184,8 @@
       <c r="F9" s="7" t="n">
         <v>1150</v>
       </c>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -5012,6 +5208,8 @@
       <c r="F10" s="7" t="n">
         <v>6246</v>
       </c>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -5034,6 +5232,8 @@
       <c r="F11" s="7" t="n">
         <v>13869</v>
       </c>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -5056,6 +5256,8 @@
       <c r="F12" s="7" t="n">
         <v>4676</v>
       </c>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -5078,6 +5280,8 @@
       <c r="F13" s="7" t="n">
         <v>1033</v>
       </c>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -5100,6 +5304,8 @@
       <c r="F14" s="7" t="n">
         <v>1111</v>
       </c>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -5122,6 +5328,8 @@
       <c r="F15" s="7" t="n">
         <v>1115</v>
       </c>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -5144,6 +5352,8 @@
       <c r="F16" s="7" t="n">
         <v>1377</v>
       </c>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -5166,6 +5376,8 @@
       <c r="F17" s="7" t="n">
         <v>2368</v>
       </c>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -5188,6 +5400,8 @@
       <c r="F18" s="7" t="n">
         <v>10820</v>
       </c>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -5210,6 +5424,8 @@
       <c r="F19" s="7" t="n">
         <v>19212</v>
       </c>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -5232,6 +5448,8 @@
       <c r="F20" s="7" t="n">
         <v>14216</v>
       </c>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -5254,6 +5472,8 @@
       <c r="F21" s="7" t="n">
         <v>9226</v>
       </c>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -5276,6 +5496,8 @@
       <c r="F22" s="7" t="n">
         <v>9676</v>
       </c>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -5298,6 +5520,8 @@
       <c r="F23" s="7" t="n">
         <v>16267</v>
       </c>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -5320,6 +5544,8 @@
       <c r="F24" s="7" t="n">
         <v>19913</v>
       </c>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -5342,6 +5568,8 @@
       <c r="F25" s="7" t="n">
         <v>20146</v>
       </c>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -5364,6 +5592,8 @@
       <c r="F26" s="7" t="n">
         <v>20904</v>
       </c>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -5386,6 +5616,8 @@
       <c r="F27" s="7" t="n">
         <v>13251</v>
       </c>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -5408,6 +5640,8 @@
       <c r="F28" s="7" t="n">
         <v>8252</v>
       </c>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -5430,6 +5664,8 @@
       <c r="F29" s="7" t="n">
         <v>11138</v>
       </c>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -5452,6 +5688,8 @@
       <c r="F30" s="7" t="n">
         <v>19750</v>
       </c>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -5474,6 +5712,8 @@
       <c r="F31" s="7" t="n">
         <v>19311</v>
       </c>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -5496,6 +5736,8 @@
       <c r="F32" s="7" t="n">
         <v>12709</v>
       </c>
+      <c r="G32" s="7" t="n"/>
+      <c r="H32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -5518,6 +5760,8 @@
       <c r="F33" s="7" t="n">
         <v>12084</v>
       </c>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -5540,6 +5784,8 @@
       <c r="F34" s="7" t="n">
         <v>12924</v>
       </c>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -5562,6 +5808,8 @@
       <c r="F35" s="7" t="n">
         <v>14373</v>
       </c>
+      <c r="G35" s="7" t="n"/>
+      <c r="H35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -5584,6 +5832,8 @@
       <c r="F36" s="7" t="n">
         <v>10410</v>
       </c>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -5606,6 +5856,8 @@
       <c r="F37" s="7" t="n">
         <v>10442</v>
       </c>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -5628,6 +5880,8 @@
       <c r="F38" s="7" t="n">
         <v>13075</v>
       </c>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -5650,6 +5904,8 @@
       <c r="F39" s="7" t="n">
         <v>14116</v>
       </c>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -5672,6 +5928,8 @@
       <c r="F40" s="7" t="n">
         <v>18691</v>
       </c>
+      <c r="G40" s="7" t="n"/>
+      <c r="H40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -5694,6 +5952,8 @@
       <c r="F41" s="7" t="n">
         <v>21047</v>
       </c>
+      <c r="G41" s="7" t="n"/>
+      <c r="H41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -5716,6 +5976,8 @@
       <c r="F42" s="7" t="n">
         <v>30610</v>
       </c>
+      <c r="G42" s="7" t="n"/>
+      <c r="H42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -5738,6 +6000,8 @@
       <c r="F43" s="7" t="n">
         <v>33029</v>
       </c>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -5760,6 +6024,8 @@
       <c r="F44" s="7" t="n">
         <v>26109</v>
       </c>
+      <c r="G44" s="7" t="n"/>
+      <c r="H44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -5782,6 +6048,8 @@
       <c r="F45" s="7" t="n">
         <v>28711</v>
       </c>
+      <c r="G45" s="7" t="n"/>
+      <c r="H45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -5804,6 +6072,8 @@
       <c r="F46" s="7" t="n">
         <v>21532</v>
       </c>
+      <c r="G46" s="7" t="n"/>
+      <c r="H46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -5826,6 +6096,8 @@
       <c r="F47" s="7" t="n">
         <v>21049</v>
       </c>
+      <c r="G47" s="7" t="n"/>
+      <c r="H47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -5848,6 +6120,8 @@
       <c r="F48" s="7" t="n">
         <v>23330</v>
       </c>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -5870,6 +6144,8 @@
       <c r="F49" s="7" t="n">
         <v>22952</v>
       </c>
+      <c r="G49" s="7" t="n"/>
+      <c r="H49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -5892,6 +6168,8 @@
       <c r="F50" s="7" t="n">
         <v>25494</v>
       </c>
+      <c r="G50" s="7" t="n"/>
+      <c r="H50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -5914,6 +6192,8 @@
       <c r="F51" s="7" t="n">
         <v>21006</v>
       </c>
+      <c r="G51" s="7" t="n"/>
+      <c r="H51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -5936,6 +6216,12 @@
       <c r="F52" s="7" t="n">
         <v>15955</v>
       </c>
+      <c r="G52" s="7" t="n">
+        <v>216603</v>
+      </c>
+      <c r="H52" s="7" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -5958,6 +6244,12 @@
       <c r="F53" s="7" t="n">
         <v>18492</v>
       </c>
+      <c r="G53" s="7" t="n">
+        <v>206420</v>
+      </c>
+      <c r="H53" s="7" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -5980,6 +6272,12 @@
       <c r="F54" s="7" t="n">
         <v>41969</v>
       </c>
+      <c r="G54" s="7" t="n">
+        <v>171964</v>
+      </c>
+      <c r="H54" s="7" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -6002,6 +6300,12 @@
       <c r="F55" s="7" t="n">
         <v>39967</v>
       </c>
+      <c r="G55" s="7" t="n">
+        <v>183635</v>
+      </c>
+      <c r="H55" s="7" t="n">
+        <v>140</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -6024,6 +6328,12 @@
       <c r="F56" s="7" t="n">
         <v>34986</v>
       </c>
+      <c r="G56" s="7" t="n">
+        <v>182983</v>
+      </c>
+      <c r="H56" s="7" t="n">
+        <v>131</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -6046,6 +6356,12 @@
       <c r="F57" s="7" t="n">
         <v>35430</v>
       </c>
+      <c r="G57" s="7" t="n">
+        <v>194202</v>
+      </c>
+      <c r="H57" s="7" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -6068,6 +6384,12 @@
       <c r="F58" s="7" t="n">
         <v>58425</v>
       </c>
+      <c r="G58" s="7" t="n">
+        <v>176299</v>
+      </c>
+      <c r="H58" s="7" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -6090,6 +6412,12 @@
       <c r="F59" s="7" t="n">
         <v>144747</v>
       </c>
+      <c r="G59" s="7" t="n">
+        <v>191000</v>
+      </c>
+      <c r="H59" s="7" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -6112,6 +6440,12 @@
       <c r="F60" s="7" t="n">
         <v>134172</v>
       </c>
+      <c r="G60" s="7" t="n">
+        <v>195865</v>
+      </c>
+      <c r="H60" s="7" t="n">
+        <v>182</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -6134,6 +6468,12 @@
       <c r="F61" s="7" t="n">
         <v>115908</v>
       </c>
+      <c r="G61" s="7" t="n">
+        <v>272403</v>
+      </c>
+      <c r="H61" s="7" t="n">
+        <v>216</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -6155,6 +6495,12 @@
       </c>
       <c r="F62" s="7" t="n">
         <v>20815</v>
+      </c>
+      <c r="G62" s="7" t="n">
+        <v>339320</v>
+      </c>
+      <c r="H62" s="7" t="n">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>